<commit_message>
[Batch] removed error headers from preview data and personal details from files
</commit_message>
<xml_diff>
--- a/tests/Functional/Batch/files/input.xlsx
+++ b/tests/Functional/Batch/files/input.xlsx
@@ -43,7 +43,7 @@
     <t>test</t>
   </si>
   <si>
-    <t>sourin.sutradhar@gmail.com</t>
+    <t>mhobbes09@gmail.com</t>
   </si>
   <si>
     <t>test payment link</t>
@@ -162,8 +162,8 @@
       <c r="C2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="1">
-        <v>7.829459269E9</v>
+      <c r="D2" s="2">
+        <v>7.0E9</v>
       </c>
       <c r="E2" s="2">
         <v>100.0</v>
@@ -184,8 +184,8 @@
       <c r="C3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="1">
-        <v>7.829459269E9</v>
+      <c r="D3" s="2">
+        <v>7.0E9</v>
       </c>
       <c r="E3" s="2">
         <v>1.0</v>
@@ -208,8 +208,8 @@
       <c r="C4" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="1">
-        <v>7.829459269E9</v>
+      <c r="D4" s="2">
+        <v>7.0E9</v>
       </c>
       <c r="E4" s="2">
         <v>200.0</v>

</xml_diff>